<commit_message>
Daily job report: 2026-03-01
</commit_message>
<xml_diff>
--- a/reports/2026-03-01_jobs.xlsx
+++ b/reports/2026-03-01_jobs.xlsx
@@ -464,13 +464,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="49" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -531,17 +531,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Manager / Senior Manager (Strategy), SPR, SNDG</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Welsbach Group</t>
+          <t>Ministry of Digital Development and Information</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi, India</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>The job title is a close match to the candidate's target roles, the location is preferred, and some skills may overlap, making it an excellent match.</t>
+          <t>The Manager / Senior Manager (Strategy) role at Ministry of Digital Development and Information is an excellent match, given the alignment of the role with the candidate's target roles, skills, and location.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -570,17 +570,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Product Management IC4</t>
+          <t>Director Product Management</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>The role of Product Management IC4 at Microsoft aligns with the candidate's target roles and skills in product management, and the location is also preferred by the candidate.</t>
+          <t>The job title aligns with the candidate's target role of Product Management, the company is a major player in the industry, and the location is within the candidate's preferred region.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -601,11 +601,7 @@
           <t>Apply Here</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -613,17 +609,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Director Product Management</t>
+          <t>Principal Product Manager - Dynamics 365 Contact Center</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Sydney, New South Wales, Australia</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -632,11 +628,11 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target role of Product Management, and the location is preferred.</t>
+          <t>The role of Principal Product Manager - Dynamics 365 Contact Center aligns with the candidate's target roles and skills, but the location is not specified as preferred.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -671,11 +667,11 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target role of Product Management, and the location is preferred.</t>
+          <t>The job title aligns with the candidate's target role of Product Management, the company is a major player in the industry, and the location is within the candidate's preferred region, with a focus on product knowledge.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -710,11 +706,11 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target role of Product Management, and the location is preferred.</t>
+          <t>The job title aligns with the candidate's target role of Product Management, the company is a major player in the industry, and the location is within the candidate's preferred region, with a focus on risk and compliance that could utilize the candidate's governance and compliance skills.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -749,11 +745,11 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target role of Product Management, and the location is preferred.</t>
+          <t>The job title aligns with the candidate's target role of Product Management, the company is a major player in the industry, and the location is within the candidate's preferred region, with a focus on product knowledge that could be a good fit for the candidate's skills and experience.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -769,17 +765,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Group Product Manager</t>
+          <t>Product Manager, Workforce Management, Platform Responsibility</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Adobe</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Noida, Uttar Pradesh, India</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -792,7 +788,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target roles, the location matches the candidate's preferred location, and the company is a well-known brand.</t>
+          <t>The Product Manager role at TikTok is an excellent match for the candidate, given the alignment of the role with their target roles and skills, and the location being in Singapore.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -808,17 +804,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Interesting Job Opportunity: Xcelore - Product Owner</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Xcelore</t>
+          <t>Flipkart</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Noida, Uttar Pradesh, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -831,7 +827,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target roles, the location matches the candidate's preferred location, and the job description implies a good fit for the candidate's skills.</t>
+          <t>The job title and company align with the candidate's target role and industry experience, and the location is within the candidate's preferred region.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -847,17 +843,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Senior Manager/Director Product Management - Missionforce</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>SOTI</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -870,7 +866,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>The job title is a close match to the candidate's target roles, the location is preferred, and some skills may overlap, making it an excellent match, but slightly less than job 8 due to company or industry differences.</t>
+          <t>The Senior Manager/Director Product Management role at Salesforce is an excellent match for the candidate, aligning with their target roles and skills in product management and digital transformation strategy.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -886,17 +882,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Technical Program Management IC4</t>
+          <t>CTO (Co-Founder) — AI Startup (WARTENS)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>WARTENS LTD</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -909,7 +905,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>The role of Technical Program Management IC4 at Microsoft aligns with the candidate's skills in project management and digital transformation, and the location is also preferred by the candidate.</t>
+          <t>The CTO role at WARTENS LTD is an excellent match for the candidate, given their skills in digital transformation strategy, AI development, and experience in managing projects and stakeholders.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -925,17 +921,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Growth Marketing (GTM) Intern</t>
+          <t>Senior Product Manager-eCommerce Platform</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Scalient</t>
+          <t>Restive</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi, India</t>
+          <t>Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -948,7 +944,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>The Growth Marketing Intern role at Scalient is an excellent match, as it includes marketing which is one of the candidate's target roles, the location is in India, and the company is in the digital transformation space.</t>
+          <t>The role of Senior Product Manager-eCommerce Platform aligns with the candidate's target roles and skills, but the location is not specified as preferred.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -959,277 +955,281 @@
       <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Product Owner</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Red Hat</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>The role of Product Owner at Red Hat is a good match as it aligns with the candidate's target roles and skills, and the location is preferred.</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Associate Product Manager</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>EY</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Melbourne, Victoria, Australia</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>The role of Associate Product Manager aligns with the candidate's target role of Product Management, and the location could be preferred.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Associate UI/UX Designer in Noida</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Aadinath UR Homes Infra Realtech</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Product manager</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Pepperstone</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Melbourne, Victoria, Australia</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>The role of Product Manager aligns with the candidate's target role of Product Management, and the location could be preferred.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Group Product Manager</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Noida, Uttar Pradesh, India</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>The role of Associate UI/UX Designer is a good match, and the location is preferred, the required skills such as UI/UX Wireframing align with the candidate's profile.</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Sr Product Associate - CCB Product</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>JPMorganChase</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>The role of Group Product Manager aligns with the candidate's target roles and skills, and the location is in India, which may be preferred given the candidate's education and lack of specified locations.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Interesting Job Opportunity: Xcelore - Product Owner</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Xcelore</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Noida, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>The role of Product Owner aligns with the candidate's target roles and skills, and the location is in India, which may be preferred given the candidate's education and lack of specified locations.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Lead, Software Engineering (AI)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Bain &amp; Company</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Gurugram, Haryana, India</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>The Lead, Software Engineering (AI) role at Bain &amp; Company is an excellent match for SUSHANT BHAT, as it involves AI development and software engineering, aligning with his skills and experience in Agentic AI Development and digital transformation.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Product Management IC4</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>The role of Sr Product Associate at JPMorganChase aligns with the candidate's target roles and skills in product management, and the location is also preferred by the candidate.</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Sales and Marketing Internship in Delhi (Hybrid)</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>KaroStartup</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Delhi, India</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>The Sales and Marketing Internship at KaroStartup is a good match, as it includes marketing which is one of the candidate's target roles and the location is in India, but it's an internship.</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Marketing Intern</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Sanyukt Organisation</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Delhi, India</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>The Marketing Intern role at Sanyukt Organisation is a good match, as it includes marketing which is one of the candidate's target roles and the location is in India, but it's an internship.</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Manager / Senior Manager (Strategy), SPR, SNDG</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Ministry of Digital Development and Information</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Singapore, Singapore</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>The job title aligns with the candidate's target role of digital transformation strategy, but the location is outside of the preferred location of India. The candidate's skills in strategy and digital transformation are highly relevant to the role.</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>The role of Product Management IC4 at Microsoft is a strong match for SUSHANT BHAT's skills and target roles, particularly in Product Management.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Flipkart</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Bengaluru, Karnataka, India</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>LinkedIn</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>60</v>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>The job is at a preferred location, and the company is a well-known firm, but the job title is not explicitly mentioned, so it's a good match.</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Apply Here</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Senior Manager/Director Product Management - Missionforce</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>The Senior Manager/Director Product Management role at Salesforce aligns well with SUSHANT BHAT's skills and experience in Product Management and Digital Transformation Strategy.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -1237,17 +1237,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>CTO (Co-Founder) — AI Startup (WARTENS)</t>
+          <t>Business &amp; Product Management, Investments - MariBank</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>WARTENS LTD</t>
+          <t>MariBank Singapore</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1256,11 +1256,11 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>The role of CTO at WARTENS is a good match as it aligns with some of the candidate's skills, but the job title and company type may not be the best fit.</t>
+          <t>The role of Business &amp; Product Management at MariBank aligns with the candidate's target roles and skills, but the location is not specified as preferred by the candidate, resulting in a good match score.</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -1276,17 +1276,17 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Founders Associate Intern</t>
+          <t>Senior Product Manager - A26032</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>OctaSence</t>
+          <t>Activate Interactive</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1295,11 +1295,11 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>The job title and location align with the candidate's preferences, and the role of Founders Associate Intern may involve some aspects of product management, digital transformation, or business solution, which are primary target roles for the candidate. The candidate's skills in digital transformation strategy and product management may be applicable to this job.</t>
+          <t>The job title aligns with the candidate's target role of Product Management, but the location is not preferred and some skills may not be directly applicable.</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1315,17 +1315,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Associate Product Manager</t>
+          <t>Product Owner</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>EY</t>
+          <t>Red Hat</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Melbourne, Victoria, Australia</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1334,11 +1334,11 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>The job is an associate product manager role which aligns with the candidate's target roles, but the location is not preferred.</t>
+          <t>The Product Owner role at Red Hat is a good match for the candidate, aligning with their skills in product management, stakeholder management, and project management.</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -1354,17 +1354,17 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Product manager</t>
+          <t>Senior Manager or Manager, AI Engineering</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Pepperstone</t>
+          <t>The Walt Disney Company</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Melbourne, Victoria, Australia</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>The job is a product manager role which aligns with the candidate's target roles, but the location is not preferred.</t>
+          <t>The Senior Manager or Manager, AI Engineering role at The Walt Disney Company is a good match for the candidate, given their skills in AI development, digital transformation strategy, and experience in managing projects and stakeholders.</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1393,17 +1393,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Sr. Director, Product Management (Platform &amp; Core Products)</t>
+          <t>Associate UI/UX Designer in Noida</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>HighLevel</t>
+          <t>Aadinath UR Homes Infra Realtech</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Delhi, Delhi, India</t>
+          <t>Noida, Uttar Pradesh, India</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1412,11 +1412,11 @@
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>The job title matches the candidate's target roles, the location matches the candidate's preferred location, but the job is a senior role that may require more experience than the candidate has.</t>
+          <t>The role of Associate UI/UX Designer aligns with the candidate's skills in UI/UX wireframing, and the location is also preferred, but the job title does not exactly match the target roles.</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -1432,17 +1432,17 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Saleforce Business Analyst</t>
+          <t>Sr Product Associate - CCB Product</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>TELUS Digital</t>
+          <t>JPMorganChase</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Noida, Uttar Pradesh, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1451,11 +1451,11 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>The role of Saleforce Business Analyst is a good match, and the location is preferred, some of the required skills such as CRM Systems may align with the candidate's profile.</t>
+          <t>The Sr Product Associate role at JPMorganChase is a good match for SUSHANT BHAT, but may be a slightly junior role given his experience</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -1471,17 +1471,17 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Lead, Software Engineering (AI)</t>
+          <t>Technical Program Management IC4</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Bain &amp; Company</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Gurugram, Haryana, India</t>
+          <t>Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1490,11 +1490,11 @@
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>The job location is preferred, and the title includes AI, which is one of the candidate's skills, but the job description does not fully align with the candidate's target roles, making it a good match.</t>
+          <t>The Technical Program Management IC4 role at Microsoft has some overlap with SUSHANT BHAT's skills, particularly in Project Management and Digital Transformation Strategy.</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -1510,17 +1510,17 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>AI Software Development Lead</t>
+          <t>Sales and Marketing Internship in Delhi (Hybrid)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Gloroots AI</t>
+          <t>KaroStartup</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Gurgaon, Haryana, India</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1529,11 +1529,11 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>The job location is preferred, and the title includes AI, which is one of the candidate's skills, making it a good match, but the job description does not fully align with the candidate's target roles.</t>
+          <t>The role of Sales and Marketing Internship has some overlap with the candidate's skills in Market Research, Competitor Analysis, and Stakeholder Management, and is in a related field, resulting in a good match.</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -1549,17 +1549,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Product Director - Customer Account Enablement Services</t>
+          <t>Marketing Intern</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>JPMorganChase</t>
+          <t>Sanyukt Organisation</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1568,11 +1568,11 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>The role of Product Director at JPMorganChase partially aligns with the candidate's target roles, but the director level may require more experience than the candidate has.</t>
+          <t>The role of Marketing Intern aligns with the candidate's target role of Product Marketing Intern and has some overlap with the candidate's skills in Market Research and Competitor Analysis, resulting in a good match.</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -1588,17 +1588,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Hr and marketing internship</t>
+          <t>Director, External Manufacturing</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Lernx</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Bahadurgarh, Haryana, India</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>The Hr and marketing internship at Lernx is a partial match, as it includes marketing which is one of the candidate's target roles, but the location is not preferred and it's an internship.</t>
+          <t>The Director, External Manufacturing role at AbbVie is a good match, as the role aligns with some of the candidate's skills, and the location is in Singapore, but the industry may not be the best fit.</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -1620,6 +1620,591 @@
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Product Manager / Director, Options Trading</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Singapore, Singapore</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>The job title aligns with the candidate's target role of Product Management, but the location is not preferred and some skills may not be directly applicable to options trading.</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Senior Program Manager</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>The role of Senior Program Manager at Oracle aligns with the candidate's skills in project management and stakeholder management, but may not fully utilize their digital transformation strategy skills.</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Founders Associate Intern</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>OctaSence</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>The role of Founders Associate Intern has some overlap with the candidate's target roles, such as Product Management and Digital Transformation, and the location matches.</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Sr. Product Success Manager (for product managers who want to guide other product teams)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Aha!</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>The role of Sr Product Success Manager aligns with the candidate's target role of Product Management, but the location is not specific.</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Product Manager - Procare</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Stryker</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Sydney, New South Wales, Australia</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>The role of Product Manager aligns with the candidate's target roles and skills, but the location is not specified as preferred.</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Product Manager, Australia</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Bendigo Advertiser</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Bar Beach, New South Wales, Australia</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>The role of Product Manager aligns with the candidate's target roles and skills, but the location is not specified as preferred.</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Product Success Manager (for product managers who want to guide other product teams)</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Aha!</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>The role of Product Success Manager aligns with the candidate's target roles and skills, but the location is not specified as preferred.</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Sr. Director, Product Management (Platform &amp; Core Products)</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>HighLevel</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Delhi, Delhi, India</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>The role of Sr. Director, Product Management aligns with the candidate's target roles, but it may require more experience than the candidate has, and the location is in India, which may be preferred.</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Cloud Account Executive - Manufacturing, Automotive</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Gurgaon, Haryana, India</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>The role of Cloud Account Executive has some alignment with the candidate's skills, particularly in areas like digital transformation and stakeholder management, and the location is also preferred.</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Saleforce Business Analyst</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>TELUS Digital</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Noida, Uttar Pradesh, India</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>The role of Salesforce Business Analyst at TELUS Digital is a good match for SUSHANT BHAT as it involves digital transformation and business analysis, aligning with his skills and experience, although the job title does not exactly match his target roles.</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Product Director - Customer Account Enablement Services</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>JPMorganChase</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>The Product Director role at JPMorganChase has some overlap with SUSHANT BHAT's skills, but may require more seniority or different expertise.</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Readiness Program Senior Manager- NPI</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>The Readiness Program Senior Manager role at Salesforce has some overlap with the candidate's skills in Project Management, Stakeholder Management, and Governance &amp; Compliance Alignment, making it a good match.</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Intern, Hospitality Marketing</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Marina Bay Sands</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Singapore, Singapore</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>The role of Intern, Hospitality Marketing aligns with the candidate's target role of Product Marketing Intern and has some overlap with the candidate's skills in Market Research and Competitor Analysis, resulting in a good match.</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Marketing Trainee(Travel Opportunity)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Polo Marketing Group</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>The role of Marketing Trainee aligns with the candidate's target role of Product Marketing Intern and has some overlap with the candidate's skills in Market Research and Competitor Analysis, resulting in a good match.</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>✨📢 (TRAINING PROVIDED) BRAND MARKETING TRAINEE 😇🌈</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Altius Org</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Singapore, Singapore</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>The role of BRAND MARKETING TRAINEE aligns with the candidate's target role of Product Marketing Intern and has some overlap with the candidate's skills in Market Research and Competitor Analysis, resulting in a good match.</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Apply Here</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1651,6 +2236,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1665,7 +2265,7 @@
   <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1708,7 +2308,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6"/>
@@ -1726,7 +2326,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9"/>
@@ -1744,53 +2344,53 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Hyderabad, Telangana, India</t>
+          <t xml:space="preserve">  Singapore, Singapore</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Noida, Uttar Pradesh, India</t>
+          <t xml:space="preserve">  Hyderabad, Telangana, India</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  New Delhi, Delhi, India</t>
+          <t xml:space="preserve">  Noida, Uttar Pradesh, India</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gurgaon, Haryana, India</t>
+          <t xml:space="preserve">  Melbourne, Victoria, Australia</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Delhi, India</t>
+          <t xml:space="preserve">  Sydney, New South Wales, Australia</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1800,7 +2400,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Melbourne, Victoria, Australia</t>
+          <t xml:space="preserve">  Delhi, India</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1810,17 +2410,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Singapore, Singapore</t>
+          <t xml:space="preserve">  Australia</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Delhi, Delhi, India</t>
+          <t xml:space="preserve">  Gurugram, Haryana, India</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1830,7 +2430,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Gurugram, Haryana, India</t>
+          <t xml:space="preserve">  Bar Beach, New South Wales, Australia</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1858,41 +2458,41 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Microsoft</t>
+          <t xml:space="preserve">  Salesforce</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  JPMorganChase</t>
+          <t xml:space="preserve">  Microsoft</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Welsbach Group</t>
+          <t xml:space="preserve">  JPMorganChase</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Adobe</t>
+          <t xml:space="preserve">  Aha!</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>